<commit_message>
HQ: park hours sheet gets an hours-only tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015sd9rGiF55g53SvUATRP26
</commit_message>
<xml_diff>
--- a/.claude/build/research/KPC_Park_Hours_worklist.xlsx
+++ b/.claude/build/research/KPC_Park_Hours_worklist.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KY parks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Hours + fees (40)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Hours only (67)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -539,6 +540,13 @@
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Rules: official pages only (parks.ky.gov, eec.ky.gov, fw.ky.gov, nps.gov, fs.usda.gov, fws.gov, the park's own site). Only what the page says. Not there = leave it empty and write NOT ON PAGE in Status. No new tabs or columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TAB 2 "Hours only": after the first tab is done, do these the same way, but HOURS ONLY (these parks are free, skip the fee). Same Status rule: start at the first row with an empty Status.</t>
         </is>
       </c>
     </row>
@@ -1693,4 +1701,1776 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Park ref</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Park name</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Our link</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Hours (YOU)</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Link: exact page (YOU)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Status (YOU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>EXAMPLE</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Example Lake State Park</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/example</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Grounds 06:00-22:00 Eastern</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/example/hours</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>US-1273</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Barren River Lake State Park</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/lucas/parks/resort/barren-river-lake-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr"/>
+      <c r="F3" s="8" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>US-1274</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Blue Licks Battlefield State Park</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/carlisle/parks/historic/blue-licks-battlefield-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>US-3781</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Breaks Interstate State Park</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.breakspark.com/</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>US-1275</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Buckhorn Lake State Park</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>https://next.pota.app/park/US-1275</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>US-1251</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Carr Creek State Park</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>https://next.pota.app/park/US-1251</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>US-1276</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Carter Caves State Park</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/olive-hill/parks/resort/carter-caves-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>US-1277</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Cumberland Falls State Park</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/corbin/parks/resort/cumberland-falls-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>US-1278</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Dale Hollow State Park</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/burkesville/parks/resort/dale-hollow-lake-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>US-1254</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>E.P. 'Tom' Sawyer State Park</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/explore/e-p-tom-sawyer-state-park-7810</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>US-1257</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>General Burnside State Park</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/burnside/parks/recreation/general-burnside-island-state-park</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>US-1279</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>General Butler State Park</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/carrollton/parks/historic/general-butler-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>US-1258</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Grayson Lake State Park</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/olive-hill/parks/recreation/grayson-lake-state-park</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>US-1280</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Greenbo Lake State Park</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/ashland/parks/historic/greenbo-lake-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>US-1281</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Jenny Wiley State Park</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/prestonsburg/parks/resort/jenny-wiley-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>US-1282</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Kenlake State Park</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/hardin/parks/resort/kenlake-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>US-1283</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Kentucky Dam Village State Park</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/gilbertsville/parks/resort/kentucky-dam-village-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>US-1261</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Kincaid Lake State Park</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/falmouth/parks/recreation/kincaid-lake-state-park</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>US-1262</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Kingdom Come State Park</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/cumberland/parks/recreation/kingdom-come-state-park</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr"/>
+      <c r="F20" s="8" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>US-1284</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Lake Barkley State Park</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/cadiz/parks/resort/lake-barkley-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr"/>
+      <c r="F21" s="8" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>US-1285</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Lake Cumberland State Park</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/jamestown/parks/resort/lake-cumberland-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>US-1263</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Lake Malone State Park</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/dunmor/parks/recreation/lake-malone-state-park</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr"/>
+      <c r="F23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>US-1264</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Levi Jackson Wilderness Road State Park</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>https://levijacksonpark.com/</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>US-1266</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Mineral Mounds State Park</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/eddyville/parks/recreation/mineral-mound-state-park</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr"/>
+      <c r="F25" s="8" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>US-1267</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>My Old Kentucky Home State Park</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/bardstown/parks/historic/my-old-kentucky-home-state-park</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>US-1286</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Natural Bridge State Park</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/slade/parks/resort/natural-bridge-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr"/>
+      <c r="F27" s="8" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>US-1268</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Nolin Lake State Park</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/mammoth-cave/parks/recreation/nolin-lake-state-park</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr"/>
+      <c r="F28" s="8" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>US-1270</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Paintsville Lake State Park</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/staffordsville/parks/recreation/paintsville-lake-state-park</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr"/>
+      <c r="F29" s="8" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>US-1287</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Pennyrile Forest State Park</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/dawson-springs/parks/resort/pennyrile-forest-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr"/>
+      <c r="F30" s="8" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>US-1288</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Pine Mountain State Park</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/pineville/parks/resort/pine-mountain-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr"/>
+      <c r="F31" s="8" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>US-1289</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Rough River Dam State Park</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/falls-rough/parks/resort/rough-river-dam-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr"/>
+      <c r="F32" s="8" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>US-1271</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Taylorsville Lake State Park</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/mount-eden/parks/recreation/taylorsville-lake-state-park</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr"/>
+      <c r="F33" s="8" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>US-1272</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Yatesville Lake State Park</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>State Park</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/louisa/parks/recreation/yatesville-lake-state-park</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr"/>
+      <c r="F34" s="8" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>US-7966</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Bad Branch State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Bad-Branch.aspx</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr"/>
+      <c r="F35" s="8" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>US-12971</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Bat Cave State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Carter-Caves.aspx</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr"/>
+      <c r="F36" s="8" t="inlineStr"/>
+      <c r="G36" s="8" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>US-7956</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Beargrass Creek State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Beargrass-Creek.aspx</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr"/>
+      <c r="F37" s="8" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>US-7954</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Blackacre State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Blackacre.aspx</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr"/>
+      <c r="F38" s="8" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>US-7967</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Blanton Forest State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Blanton-Forest.aspx</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr"/>
+      <c r="F39" s="8" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>US-7965</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Brigadoon State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Brigadoon.aspx</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr"/>
+      <c r="F40" s="8" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>US-12972</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Cascade Caverns State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>https://opengisdata.ky.gov/datasets/ky-knp-state-nature-preserves/explore?location=38.354945%2C-83.108279%2C14.97</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr"/>
+      <c r="F41" s="8" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>US-7960</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Crooked Creek State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Crooked-Creek.aspx</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr"/>
+      <c r="F42" s="8" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>US-7968</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>E. Lucy Braun State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/E.-Lucy-Braun.aspx</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr"/>
+      <c r="F43" s="8" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>US-12752</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Green River State Natural Area</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Rush-Island-Bottoms.aspx</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr"/>
+      <c r="F44" s="8" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>US-7957</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Hall-Hill/Vernon-Douglas State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Vernon-Douglas.aspx</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr"/>
+      <c r="F45" s="8" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>US-7961</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Jesse Stuart State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Jesse-Stuart.aspx</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr"/>
+      <c r="F46" s="8" t="inlineStr"/>
+      <c r="G46" s="8" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>US-7958</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Kentucky River Palisades/Tom Dorman State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Tom-Dorman.aspx</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr"/>
+      <c r="F47" s="8" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>US-7962</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Little South Fork State Natural Area</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Burnett-WWCA.aspx</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr"/>
+      <c r="F48" s="8" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>US-7953</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Metropolis Lake State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Metropolis-Lake.aspx</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr"/>
+      <c r="F49" s="8" t="inlineStr"/>
+      <c r="G49" s="8" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>US-7963</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Pilot Knob State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Pilot-Knob.aspx</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr"/>
+      <c r="F50" s="8" t="inlineStr"/>
+      <c r="G50" s="8" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>US-7959</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Quiet Trails State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Quiet-Trails.aspx</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr"/>
+      <c r="F51" s="8" t="inlineStr"/>
+      <c r="G51" s="8" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>US-7970</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Sinking Creek State Natural Area</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Sinking-Creek.aspx</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr"/>
+      <c r="F52" s="8" t="inlineStr"/>
+      <c r="G52" s="8" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>US-7955</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Six Mile Island State Nature Preserve</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Six-Mile-Island.aspx</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr"/>
+      <c r="F53" s="8" t="inlineStr"/>
+      <c r="G53" s="8" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>US-7964</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>William H. Martin State Natural Area</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Nature Preserve</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Dr.-William-H.-Martin-WWCA.aspx</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr"/>
+      <c r="F54" s="8" t="inlineStr"/>
+      <c r="G54" s="8" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>US-7951</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Green River State Forest</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>State Forest</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Green-River-State-Forest.aspx</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr"/>
+      <c r="F55" s="8" t="inlineStr"/>
+      <c r="G55" s="8" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>US-4688</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Kentenia State Forest</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>State Forest</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Kentenia-State-Forest.aspx</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr"/>
+      <c r="F56" s="8" t="inlineStr"/>
+      <c r="G56" s="8" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>US-4689</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Kentucky Ridge State Forest</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>State Forest</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Kentucky-Ridge-State-Forest.aspx</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr"/>
+      <c r="F57" s="8" t="inlineStr"/>
+      <c r="G57" s="8" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>US-4690</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Knobs State Forest</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>State Forest</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Knobs-State-Forest-and-Wildlife-Management-Area.aspx</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr"/>
+      <c r="F58" s="8" t="inlineStr"/>
+      <c r="G58" s="8" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>US-7952</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Marrowbone State Forest</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>State Forest</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>https://fw.ky.gov/More/Documents/MarrowboneStateForestandWMA_ALL.pdf</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr"/>
+      <c r="F59" s="8" t="inlineStr"/>
+      <c r="G59" s="8" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>US-4692</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Pennyrile State Forest</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>State Forest</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/dawson-springs/parks/resort/pennyrile-forest-state-resort-park</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr"/>
+      <c r="F60" s="8" t="inlineStr"/>
+      <c r="G60" s="8" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>US-4693</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Tygarts State Forest</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>State Forest</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Tygarts-State-Forest.aspx</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr"/>
+      <c r="F61" s="8" t="inlineStr"/>
+      <c r="G61" s="8" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>US-10102</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Pine Mountain State Trail</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>https://parks.ky.gov/whitesburg/parks/recreation/pine-mountain-state-scenic-trail</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr"/>
+      <c r="F62" s="8" t="inlineStr"/>
+      <c r="G62" s="8" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>US-11181</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Sheltowee Trace National Recreation Trail</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>https://www.fs.usda.gov/wildflowers/regions/southern/SheltoweeTrace/index.shtml</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr"/>
+      <c r="F63" s="8" t="inlineStr"/>
+      <c r="G63" s="8" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>US-13598</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Beaver Lake State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=49</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr"/>
+      <c r="F64" s="8" t="inlineStr"/>
+      <c r="G64" s="8" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>US-13607</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Boltz State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=50</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr"/>
+      <c r="F65" s="8" t="inlineStr"/>
+      <c r="G65" s="8" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>US-13606</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Bullock Pen State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=51</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr"/>
+      <c r="F66" s="8" t="inlineStr"/>
+      <c r="G66" s="8" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>US-13600</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Carpenters Lake State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=39</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr"/>
+      <c r="F67" s="8" t="inlineStr"/>
+      <c r="G67" s="8" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>US-13601</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Guist Creek Lake State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=56</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr"/>
+      <c r="F68" s="8" t="inlineStr"/>
+      <c r="G68" s="8" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>US-13599</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Kingfisher Lakes State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>State Fishing Lake</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=40</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr"/>
+      <c r="F69" s="8" t="inlineStr"/>
+      <c r="G69" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>